<commit_message>
Fix MSME vendor processing and interest calculation
</commit_message>
<xml_diff>
--- a/backend/data/test-fallback-pan/Udyam_no.xlsx
+++ b/backend/data/test-fallback-pan/Udyam_no.xlsx
@@ -32,8 +32,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy\ hh:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
   <fonts count="1">
     <font>

</xml_diff>